<commit_message>
Incorporate Taiping Life 2026Q1 solvency report and Taiping Group 2025 solvency table (primary sources); recompute replenishment power
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L8aigT8rcgficjTBusL67d
</commit_message>
<xml_diff>
--- a/mof-insurer-injection-2026-09/extended/solvency_table.xlsx
+++ b/mof-insurer-injection-2026-09/extended/solvency_table.xlsx
@@ -5819,7 +5819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6093,7 +6093,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>中國太平集團→太平人壽</t>
+          <t>中國太平集團（原文）</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -6106,46 +6106,42 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2025Q4</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>≈1,643（反推）</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>≈1,146（反推）</t>
-        </is>
+          <t>2025 年末</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2046.1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1401.1</v>
       </c>
       <c r="G4" t="n">
-        <v>2639</v>
+        <v>3103.6</v>
       </c>
       <c r="H4" t="n">
-        <v>143.32</v>
+        <v>146</v>
       </c>
       <c r="I4" t="n">
-        <v>230.18</v>
+        <v>222</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>3.4%</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>6.1%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>6.1</v>
+        <v>5</v>
       </c>
       <c r="M4" t="n">
-        <v>149.4</v>
+        <v>151</v>
       </c>
       <c r="N4" t="n">
-        <v>236.3</v>
+        <v>227</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -6167,22 +6163,22 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>假設 70 億全額下沉到太平人壽；核心／最低資本由實際資本與充足率反推</t>
+          <t>集團 2025 年度信息披露報告原文；2024 末 178%/271%，一年核心溢額流失 237 億</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>中國再保險（01508）</t>
+          <t>太平人壽（原文，假設全額下沉）</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>上市公司定增內資股</t>
+          <t>集團子公司</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -6190,170 +6186,247 @@
           <t>2026Q1</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>未找到</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>未找到（Q1 單季上升 146 億）</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>未找到</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>未找到（Q1 較上季降約 102 個百分點）</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>未找到（同左）</t>
-        </is>
+      <c r="E5" t="n">
+        <v>1556.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1165.8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2614.5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>133.51</v>
+      </c>
+      <c r="I5" t="n">
+        <v>224.27</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t>4.5%</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>6.0%</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>6</v>
+      </c>
+      <c r="M5" t="n">
+        <v>139.5</v>
+      </c>
+      <c r="N5" t="n">
+        <v>230.3</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>33.27</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>0.9 倍</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>未找到</t>
-        </is>
+      <c r="Q5" t="n">
+        <v>200</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.35 倍</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026Q1 市場風險最低資本單季升 155.8 億，是充足率暴跌主因；30 億約可回補 Q1 溢額流失（142.6 億）的兩成</t>
+          <t>太平人壽 2026Q1 償付能力報告原文；保單未來盈餘計入核心已頂上限，新股本另有約 1.5～1.7 倍乘數；公司自估 2026Q2 核心 112.25%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>中國再保險（01508）</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>30</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>上市公司定增內資股</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>未找到</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>未找到（Q1 單季上升 146 億）</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>未找到</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>未找到（Q1 較上季降約 102 個百分點）</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>未找到（同左）</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>33.27</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0.9 倍</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>未找到</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>2026Q1 市場風險最低資本單季升 155.8 億，是充足率暴跌主因；30 億約可回補 Q1 溢額流失（142.6 億）的兩成</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>中國出口信用保險</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B7" t="n">
         <v>100</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>政策性公司直接注資</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>未找到</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>未找到</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>未找到</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>未找到</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>未找到</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>不分紅</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>未找到</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>2026-06 註冊資本由 271.6 億增至 461.25 億；100 億約為新註冊資本的 21.7%</t>
         </is>

</xml_diff>